<commit_message>
se actualizaron planillas de analisis en los trabajos de concurrentes
</commit_message>
<xml_diff>
--- a/metricas_realizadas/Prog-Concurrente/Analisis de metricas/Resultados_CC_MI_NLoc_Issues_Refinamientos_Token.xlsx
+++ b/metricas_realizadas/Prog-Concurrente/Analisis de metricas/Resultados_CC_MI_NLoc_Issues_Refinamientos_Token.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\metricas_realizadas\Prog-Concurrente\Analisis de metricas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07027A5C-F912-46A1-B07F-20F581BD2D1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB2BE97-1F8C-4441-B257-B0A091B90193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resultado generales" sheetId="1" r:id="rId1"/>
@@ -178,7 +178,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -272,7 +272,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -377,7 +377,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{664D3796-913A-4AD9-82BB-B70FEB278892}" type="CELLRANGE">
+                    <a:fld id="{D46AA529-ADEA-43B7-8A95-03CB84DC8CA8}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -410,7 +410,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{222533DA-5E2A-441B-9E8D-3F738B0F2F77}" type="CELLRANGE">
+                    <a:fld id="{2747F1DC-657E-4473-9993-67A18FD82EDF}" type="CELLRANGE">
                       <a:rPr lang="es-AR"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -444,7 +444,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A946C7FD-395E-4B2C-8208-577B7C6C819A}" type="CELLRANGE">
+                    <a:fld id="{351A837E-E91F-4C55-95B2-04A55B3A0C45}" type="CELLRANGE">
                       <a:rPr lang="es-AR"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -478,7 +478,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{35347BDB-4619-4F83-9746-169EAD86D45A}" type="CELLRANGE">
+                    <a:fld id="{A3FD67F4-8483-415C-8268-3745459893BB}" type="CELLRANGE">
                       <a:rPr lang="es-AR"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -512,7 +512,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E25A68F7-2A06-446A-9AA3-784756103393}" type="CELLRANGE">
+                    <a:fld id="{0A7D3CA7-5670-4271-B832-022CFA3DA675}" type="CELLRANGE">
                       <a:rPr lang="es-AR"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -546,7 +546,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CE6F5E4C-5562-44DC-B9FA-9D823C47386D}" type="CELLRANGE">
+                    <a:fld id="{6E8C7278-647D-4129-9A77-728C2F5FC592}" type="CELLRANGE">
                       <a:rPr lang="es-AR"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -580,7 +580,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E8C91F3B-7E9A-44DE-BA98-77010BF98074}" type="CELLRANGE">
+                    <a:fld id="{2C210B25-5F27-4EF4-B448-D28952EFD81B}" type="CELLRANGE">
                       <a:rPr lang="es-AR"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -614,7 +614,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{224A96F9-3819-459C-932D-14C8A877A6C2}" type="CELLRANGE">
+                    <a:fld id="{7669B00E-F8B7-4261-A831-E0192668C580}" type="CELLRANGE">
                       <a:rPr lang="es-AR"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -654,7 +654,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{46D90C85-3DCD-4797-B1D6-331C4AD3F3D9}" type="CELLRANGE">
+                    <a:fld id="{AF7E9C8D-A791-4CDD-8FDF-10FD973E11B0}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -687,7 +687,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8537AEB5-5FF5-451D-BA17-1A01C8E3DC60}" type="CELLRANGE">
+                    <a:fld id="{7136C15F-9B4E-4BC1-8785-4FA932E5F792}" type="CELLRANGE">
                       <a:rPr lang="es-AR"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3381,7 +3381,7 @@
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0">
+                <c:pt idx="0" formatCode="0.00">
                   <c:v>0.11735291922195014</c:v>
                 </c:pt>
                 <c:pt idx="1">
@@ -3621,7 +3621,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>

</xml_diff>